<commit_message>
Updates on Player Country and Date of Birth columns
</commit_message>
<xml_diff>
--- a/Data/UEFA Stats 2019_with_market_values.xlsx
+++ b/Data/UEFA Stats 2019_with_market_values.xlsx
@@ -2762,6 +2762,9 @@
       <c r="K2" t="s">
         <v>733</v>
       </c>
+      <c r="M2">
+        <v>1993</v>
+      </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
@@ -2797,6 +2800,9 @@
       <c r="K3" t="s">
         <v>734</v>
       </c>
+      <c r="M3">
+        <v>1997</v>
+      </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
@@ -2832,6 +2838,9 @@
       <c r="K4" t="s">
         <v>735</v>
       </c>
+      <c r="M4">
+        <v>1989</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
@@ -2867,6 +2876,9 @@
       <c r="K5" t="s">
         <v>736</v>
       </c>
+      <c r="M5">
+        <v>1992</v>
+      </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
@@ -2901,6 +2913,9 @@
       </c>
       <c r="K6" t="s">
         <v>737</v>
+      </c>
+      <c r="M6">
+        <v>1990</v>
       </c>
     </row>
     <row r="7" spans="1:13">

</xml_diff>